<commit_message>
Place Jutafol 145 Al above CD under mineral wool
Move the slope vapour foil from the NH/GKF pack to the attic face of
the CD (matching the rest of the house), drop the variable-foil option,
and finish the šikmina label column, Nonius hang length, and soffit ducts.

Co-authored-by: Petr Sima <ptea.sima@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -793,56 +793,60 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="n">
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Parozábrana</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Parotěsná fólie</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>≈ 1 mm (model)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Reflexní parozábrana Al</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al (JUTA; retail N AL 170 Speciál 75 m²)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Al reflex · Sd vysoké · role 1,5×50 m</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="9" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno: typ / Sd / systém pásek.</t>
+      <c r="J6" s="10" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>2791</v>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m². S rezervou 10 % ≈ 78.1 m² ≈ 2× role 75 m². Přesahy: JUTAFOL SP AL / SP 1.</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1268,7 @@
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="16" t="n">
-        <v>58179</v>
+        <v>60970</v>
       </c>
       <c r="L15" s="15" t="n"/>
       <c r="M15" s="15" t="n"/>
@@ -1272,7 +1276,7 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Parozábrana; Výplň dutiny / mezi krokvemi; Krov (nosná konstrukce)</t>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Výplň dutiny / mezi krokvemi; Krov (nosná konstrukce)</t>
         </is>
       </c>
       <c r="B16" s="18" t="n"/>
@@ -1299,10 +1303,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1716,7 +1721,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>5.76</v>
+        <v>5.78</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1729,13 +1734,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>6.46</v>
+        <v>6.47</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16625</v>
+        <v>16627</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -3071,56 +3076,60 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Parozábrana</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Fólie</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>role 75 m²</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="9" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno.</t>
+      <c r="J7" s="10" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>2791</v>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou.</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3158,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>76.76000000000001</v>
+        <v>76.78</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3162,13 +3171,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>85.98</v>
+        <v>85.98999999999999</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>9963</v>
+        <v>9965</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -3892,7 +3901,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>102909</v>
+        <v>105702</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
@@ -3900,7 +3909,7 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Parozábrana; Minerální vlna (souhrn)</t>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna (souhrn)</t>
         </is>
       </c>
       <c r="B23" s="18" t="n"/>
@@ -3928,12 +3937,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Export the CD/UD soffit and the built-lattice report.
The preview model, section drawing, and material list now show the steel kastlík frame. The acoustics report leads with kitchen 625 vertical and living 1000 horizontal at the as-built wool.

Co-authored-by: Petr Sima <ptea.sima@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -1645,26 +1645,26 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Latový rošt</t>
+          <t>Rošt kastlíku</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Dřevěné latě</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40 mm</t>
+          <t>Profil CD 60×27</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Rigips R-CD 27/60/27</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>60×40 @ 625</t>
+          <t>60×27 @ 625</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1673,26 +1673,26 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>12 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>19.7</v>
+        <v>19.1</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>45</v>
+        <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>885</v>
+        <v>557</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>32 prvků (svislé + spodní).</t>
+          <t>32 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Drop CD → latový rošt</t>
+          <t>Drop CD → svislý CD</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2183,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16627</v>
+        <v>16299</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2218,9 +2218,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2418,11 +2419,11 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>60×27 @ 625</t>
+          <t>kuchyň 625 svisle + dořez; obývák 1000 + dořez</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>109.4</v>
+        <v>101.8</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2435,13 +2436,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>120.3</v>
+        <v>111.9</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3515</v>
+        <v>3270</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2450,7 +2451,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>UW detaily dle montáže — v modelu jako CD.</t>
+          <t>Lišty pod spárou: kuchyň 2000 mm, obývák 1250 a 2500 mm, na CD. UW v modelu jako CD.</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2482,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2494,13 +2495,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2705,7 +2706,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>28105</v>
+        <v>23223</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -3272,7 +3273,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>219.7</v>
+        <v>229.4</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3285,13 +3286,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>241.7</v>
+        <v>252.4</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7060</v>
+        <v>7372</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -3443,7 +3444,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3456,13 +3457,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3500,7 +3501,7 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>33.07</v>
+        <v>33.09</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -3513,7 +3514,7 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>36.38</v>
+        <v>36.4</v>
       </c>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
@@ -3524,64 +3525,64 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.63 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="n">
+          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.65 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Řezivo</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>60×40</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UD 28×27</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>UD profil</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Rigips UD (obvod kastlíku)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>28×27</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>12 %</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>885</v>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>Kastlík.</t>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>29.21</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>336</v>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3902,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>105702</v>
+        <v>100828</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>

</xml_diff>

<commit_message>
Put the shallow bass trap on the two-door kitchen gable.
The model called Y=0 the kitchen and built the 190 mm trap there, but that
wall has one sliding door. The two doors are at Y=L. Those openings stay
put. The 190 mm stack now sits on Y=L and the 450 mm stack on Y=0. The
taped coverage winner remains kitchen 625 vertical and living 1000
horizontal, and the as-built wool stays because no band moves by more than 5%.

Co-authored-by: Petr Sima <ptea.sima@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>17.3</v>
+        <v>18.4</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1677,13 +1677,13 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>19.1</v>
+        <v>20.3</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>557</v>
+        <v>592</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>32 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
+          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1905,13 +1905,13 @@
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="J11" s="12" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="I13" s="6" t="n">
-        <v>35.2</v>
+        <v>37.4</v>
       </c>
       <c r="J13" s="12" t="n">
         <v>35</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>1232</v>
+        <v>1309</v>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16299</v>
+        <v>16420</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>kuchyň 625 svisle + dořez; obývák 1000 + dořez</t>
+          <t>kuchyň (Y=L, dva posuvné, 190) 625 svisle + dořez; obývák (Y=0, jedny, 450) 1000 + dořez</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>Lišty pod spárou: kuchyň 2000 mm, obývák 1250 a 2500 mm, na CD. UW v modelu jako CD.</t>
+          <t>Lišty pod spárou: kuchyň 2000 mm na dvouposuvném štítu, obývák 1250 a 2500 mm na jednoposuvném. UW v modelu jako CD.</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Split 130.5+47.0+12.5 = 190 mm.</t>
+          <t>Split 130.5+47.0+12.5 = 190 mm. Štít se dvěma posuvnými dveřmi.</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Split 12.5+137.5+300.0 = 450 mm.</t>
+          <t>Split 12.5+137.5+300.0 = 450 mm. Štít s jedněmi posuvnými dveřmi, subwoofer v rohu u TV.</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>229.4</v>
+        <v>230.5</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3286,13 +3286,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>252.4</v>
+        <v>253.6</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7372</v>
+        <v>7407</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -3725,7 +3725,7 @@
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -3738,13 +3738,13 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="J18" s="12" t="n">
         <v>8</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -3852,13 +3852,13 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>35.2</v>
+        <v>37.4</v>
       </c>
       <c r="J20" s="12" t="n">
         <v>35</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>1232</v>
+        <v>1309</v>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
@@ -3902,7 +3902,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>100828</v>
+        <v>100949</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>

</xml_diff>

<commit_message>
Shallow bass trap on the two-door kitchen gable (#54)
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -1645,26 +1645,26 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Latový rošt</t>
+          <t>Rošt kastlíku</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Dřevěné latě</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40 mm</t>
+          <t>Profil CD 60×27</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Rigips R-CD 27/60/27</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>60×40 @ 625</t>
+          <t>60×27 @ 625</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1673,26 +1673,26 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>12 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>45</v>
+        <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>885</v>
+        <v>592</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>32 prvků (svislé + spodní).</t>
+          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Drop CD → latový rošt</t>
+          <t>Drop CD → svislý CD</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1905,13 +1905,13 @@
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="J11" s="12" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="I13" s="6" t="n">
-        <v>35.2</v>
+        <v>37.4</v>
       </c>
       <c r="J13" s="12" t="n">
         <v>35</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>1232</v>
+        <v>1309</v>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16627</v>
+        <v>16420</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2218,9 +2218,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2418,11 +2419,11 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>60×27 @ 625</t>
+          <t>kuchyň (Y=L, dva posuvné, 190) 625 svisle + dořez; obývák (Y=0, jedny, 450) 1000 + dořez</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>109.4</v>
+        <v>101.8</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2435,13 +2436,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>120.3</v>
+        <v>111.9</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3515</v>
+        <v>3270</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2450,7 +2451,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>UW detaily dle montáže — v modelu jako CD.</t>
+          <t>Lišty pod spárou: kuchyň 2000 mm na dvouposuvném štítu, obývák 1250 a 2500 mm na jednoposuvném. UW v modelu jako CD.</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2482,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2494,13 +2495,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2615,7 +2616,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Split 130.5+47.0+12.5 = 190 mm.</t>
+          <t>Split 130.5+47.0+12.5 = 190 mm. Štít se dvěma posuvnými dveřmi.</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2671,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Split 12.5+137.5+300.0 = 450 mm.</t>
+          <t>Split 12.5+137.5+300.0 = 450 mm. Štít s jedněmi posuvnými dveřmi, subwoofer v rohu u TV.</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2706,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>28105</v>
+        <v>23223</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -3272,7 +3273,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>219.7</v>
+        <v>230.5</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3285,13 +3286,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>241.7</v>
+        <v>253.6</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7060</v>
+        <v>7407</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -3443,7 +3444,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3456,13 +3457,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3500,7 +3501,7 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>33.07</v>
+        <v>33.09</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -3513,7 +3514,7 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>36.38</v>
+        <v>36.4</v>
       </c>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
@@ -3524,64 +3525,64 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.63 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="n">
+          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.65 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Řezivo</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>60×40</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UD 28×27</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>UD profil</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Rigips UD (obvod kastlíku)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>28×27</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>12 %</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>885</v>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>Kastlík.</t>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>29.21</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>336</v>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3725,7 @@
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -3737,13 +3738,13 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="J18" s="12" t="n">
         <v>8</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
@@ -3838,7 +3839,7 @@
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -3851,13 +3852,13 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>35.2</v>
+        <v>37.4</v>
       </c>
       <c r="J20" s="12" t="n">
         <v>35</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>1232</v>
+        <v>1309</v>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
@@ -3901,7 +3902,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>105702</v>
+        <v>100949</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>

</xml_diff>

<commit_message>
Obývák: 140 mm Unifit plenum, Jutafol N AL 170, hangers 200/440
Thicker plenum fills the right slope to the rafter. Foil and wool stop at the kastlík lid so the lid Z stays put.

Co-authored-by: Petr Sima <ptea.sima@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -809,12 +809,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Jutafol 145 Al (JUTA; retail N AL 170 Speciál 75 m²)</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Al reflex · Sd vysoké · role 1,5×50 m</t>
+          <t>sd &gt; 300 m · role 1,5×50 m = 75 m²</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
@@ -841,12 +841,12 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m². S rezervou 10 % ≈ 78.1 m² ≈ 2× role 75 m². Přesahy: JUTAFOL SP AL / SP 1.</t>
+          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m². S rezervou 10 % ≈ 78.1 m² ≈ 2× role 75 m². Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
@@ -975,17 +975,17 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 125 mm</t>
+          <t>Přímý závěs 200 mm DK Mont</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Rigips přímý závěs 125 mm, KB510154</t>
+          <t>Přímý závěs 200 mm DK Mont 3631100170</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>125 mm</t>
+          <t>200 mm</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
@@ -1005,19 +1005,19 @@
         <v>56.2</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>6.27</v>
+        <v>12.52</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>352</v>
+        <v>703</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>DEK KB510154 · https://www.dek.cz/produkty/detail/3630551425-primy-zaves-60-125-mm-1-00mm-100-ks-bal</t>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Kotvení z boku krokve.</t>
+          <t>Kotvení z boku krokve. Modelové svěšení 139 mm, noha 200 mm.</t>
         </is>
       </c>
     </row>
@@ -1037,12 +1037,12 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius horní 340/440 + spodní CD + 2× závlačka</t>
+          <t>Rigips Nonius horní 440 + spodní CD + 2× závlačka</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>horní 340/440 dle svěšení</t>
+          <t>horní 440 mm</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
@@ -1062,242 +1062,305 @@
         <v>70.2</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>29.1</v>
+        <v>32.07</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>2043</v>
+        <v>2251</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT horní 340 · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Svěšení otevírá se k nábytku.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="n">
+          <t>Pravá šikmina. Nejdelší svěšení v modelu 428 mm (u okapu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Výplň dutiny / mezi krokvemi</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Minerální vlna mezi krokve</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 035 160 mm</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035, 160 mm</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>160 mm · řez ~790 mm</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>75.53</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>242.24</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>18296</v>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>Plocha sklonu nad místností 77.52 m² × (775/875). Šikmina po nábytek by byla 62.89 m²; model vyplňuje pole i nad kastlíkem. Specifikace uvádí roli 1200×4000; DEK aktuálně 1200×3200 (3,84 m²).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>9b</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Minerální vlna plénum</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 035 140 mm (L) / plná mezera (P)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>L 140 mm / P 429 mm</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>23.01</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>1514.29</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>34847</v>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>Levá 140 mm. Pravá plná mezera 429 mm (140+140+150 nebo 200+220), bez vzduchu. Objem z modelu 20.92 m³ (celá vlna šikmin 31.84 − pole 10.92). Specifikace uvádí roli 140 mm 1200×4500; DEK aktuálně 1200×3700 (4,44 m²).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Zavětrování</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Ocelová páska</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>void ~80 mm + mezi krokvemi 160 mm</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>27.64</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>40×2 mm @ 45°</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I11" s="6" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="I13" s="6" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="K13" s="13" t="n">
+        <v>896</v>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>orientační ocelová páska 40×2</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Typ pásky / kotevní prvky ještě sjednotit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Krov (nosná konstrukce)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Krokve</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Stávající krov</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>100/160 @ 875</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno: typ vlny (akustika σ≈12000). Ne NaturHeld Flex.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Zavětrování</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Ocelová páska</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>40×2 mm @ 45°</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K12" s="13" t="n">
-        <v>896</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>orientační ocelová páska 40×2</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>Typ pásky / kotevní prvky ještě sjednotit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Krov (nosná konstrukce)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Krokve</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Stávající krov</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>100/160 @ 875</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="9" t="n"/>
-      <c r="L13" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>Není položka nákupu akustiky.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="15" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="16" t="n">
-        <v>60970</v>
-      </c>
-      <c r="L15" s="15" t="n"/>
-      <c r="M15" s="15" t="n"/>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Výplň dutiny / mezi krokvemi; Krov (nosná konstrukce)</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
-      <c r="I16" s="18" t="n"/>
-      <c r="J16" s="18" t="n"/>
-      <c r="K16" s="18" t="n"/>
-      <c r="L16" s="18" t="n"/>
-      <c r="M16" s="18" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="16" t="n">
+        <v>114673</v>
+      </c>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Krov (nosná konstrukce)</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
+      <c r="L17" s="18" t="n"/>
+      <c r="M17" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A15:J15"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A16:J16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -1308,6 +1371,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1448,7 +1513,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>36.38</v>
+        <v>33.92</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1461,7 +1526,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>40.01</v>
+        <v>37.31</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -1472,7 +1537,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>12.13 m² × 3,0 = 36.4 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
+          <t>11.31 m² × 3,0 = 33.9 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1566,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>30.31</v>
+        <v>28.27</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1514,7 +1579,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>33.35</v>
+        <v>31.09</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -1525,7 +1590,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>12.13 m² × 2,5 = 30.3 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
+          <t>11.31 m² × 2,5 = 28.3 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1619,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>12.13</v>
+        <v>11.31</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1567,13 +1632,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>13.58</v>
+        <v>12.66</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3612</v>
+        <v>3368</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -1597,21 +1662,21 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Minerální vlna</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>Knauf Unifit 035</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>za NH, zastaveno před potrubím</t>
+          <t>tloušťka dle modelu, před potrubím</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1624,18 +1689,18 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1.98</v>
+        <v>2.09</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: typ vlny.</t>
+          <t>Stejný výrobek jako šikminy. Tloušťka zůstává dle modelu (zastaveno před potrubím).</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1786,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>5.78</v>
+        <v>6.76</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1734,13 +1799,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>6.47</v>
+        <v>7.57</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>750</v>
+        <v>877</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -1826,12 +1891,12 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius sada</t>
+          <t>Rigips Nonius horní 440 + spodní CD + 2× závlačka</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>≈400 mm svěšení</t>
+          <t>horní 440 mm</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
@@ -1851,19 +1916,19 @@
         <v>14</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>29.1</v>
+        <v>32.07</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>409</v>
+        <v>450</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT horní 340 · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>1 závěs na krokev na rostovém CD.</t>
+          <t>1 závěs na krokev na rostovém CD. Svěšení 406 mm.</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2248,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16420</v>
+        <v>16345</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2218,10 +2283,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2364,7 +2430,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>17.88</v>
+        <v>17.18</v>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
@@ -2377,13 +2443,13 @@
         </is>
       </c>
       <c r="I3" s="9" t="n">
-        <v>20.03</v>
+        <v>19.24</v>
       </c>
       <c r="J3" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>1923</v>
+        <v>1847</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
@@ -2423,7 +2489,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>101.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2436,13 +2502,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>111.9</v>
+        <v>108.2</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3270</v>
+        <v>3160</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2482,7 +2548,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2495,13 +2561,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>37.8</v>
+        <v>36.7</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>18031</v>
+        <v>17515</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2578,12 +2644,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Minerální vlna</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>Knauf Unifit 035</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -2592,7 +2658,7 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1.14</v>
+        <v>1.09</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -2605,18 +2671,18 @@
         </is>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1.25</v>
+        <v>1.19</v>
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Split 130.5+47.0+12.5 = 190 mm. Štít se dvěma posuvnými dveřmi.</t>
+          <t>Split 130.5+47.0+12.5 = 190 mm. Štít se dvěma posuvnými dveřmi. Tloušťka dle modelu.</t>
         </is>
       </c>
     </row>
@@ -2633,12 +2699,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Minerální vlna</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>Knauf Unifit 035</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -2647,7 +2713,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2.62</v>
+        <v>2.5</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -2660,18 +2726,18 @@
         </is>
       </c>
       <c r="I8" s="6" t="n">
-        <v>2.88</v>
+        <v>2.75</v>
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Split 12.5+137.5+300.0 = 450 mm. Štít s jedněmi posuvnými dveřmi, subwoofer v rohu u TV.</t>
+          <t>Split 12.5+137.5+300.0 = 450 mm. Štít s jedněmi posuvnými dveřmi, subwoofer v rohu u TV. Tloušťka dle modelu.</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2772,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>23223</v>
+        <v>22523</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -2742,6 +2808,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2753,7 +2821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2882,7 +2950,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>249.38</v>
+        <v>246.92</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -2895,7 +2963,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>274.32</v>
+        <v>271.61</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -2906,7 +2974,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Šikminy+kastlík 83.13 m² → 249.4 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
+          <t>Šikminy+kastlík 82.31 m² → 246.9 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3003,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>207.82</v>
+        <v>205.77</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -2948,7 +3016,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>228.6</v>
+        <v>226.35</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -2959,7 +3027,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>207.8 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
+          <t>205.8 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3113,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>12.13</v>
+        <v>11.31</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -3058,13 +3126,13 @@
         </is>
       </c>
       <c r="I6" s="9" t="n">
-        <v>13.58</v>
+        <v>12.66</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>3612</v>
+        <v>3368</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -3088,12 +3156,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Jutafol 145 Al</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Jutafol 145 Al</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3125,12 +3193,12 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou.</t>
+          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>76.78</v>
+        <v>77.76000000000001</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3172,13 +3240,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>85.98999999999999</v>
+        <v>87.09</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>9965</v>
+        <v>10092</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -3216,7 +3284,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>17.88</v>
+        <v>17.18</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -3229,13 +3297,13 @@
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>20.03</v>
+        <v>19.24</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1923</v>
+        <v>1847</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
@@ -3273,7 +3341,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>230.5</v>
+        <v>227.1</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3286,13 +3354,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>253.6</v>
+        <v>249.8</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7407</v>
+        <v>7297</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -3311,22 +3379,22 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs KB510154</t>
+          <t>Přímý závěs 200 mm DK Mont</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 125</t>
+          <t>Přímý závěs 200 mm</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Rigips KB510154</t>
+          <t>DK Mont 3631100170</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>125 mm</t>
+          <t>200 mm</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
@@ -3346,19 +3414,19 @@
         <v>56.2</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>6.27</v>
+        <v>12.52</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>352</v>
+        <v>703</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK KB510154 · https://www.dek.cz/produkty/detail/3630551425-primy-zaves-60-125-mm-1-00mm-100-ks-bal</t>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Okenní šikmina.</t>
+          <t>Okenní šikmina. Svěšení 139 mm. Balení 100 ks.</t>
         </is>
       </c>
     </row>
@@ -3378,12 +3446,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius sada</t>
+          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>340/440</t>
+          <t>440</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
@@ -3403,19 +3471,19 @@
         <v>84.2</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>29.1</v>
+        <v>32.07</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>2451</v>
+        <v>2702</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT horní 340 · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Šikminy u skříní + kastlík.</t>
+          <t>Pravá šikmina + kastlík. Svěšení šikminy 428 mm, kastlík 406 mm.</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3512,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3457,13 +3525,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>37.8</v>
+        <v>36.7</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>18031</v>
+        <v>17515</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3476,113 +3544,117 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="A14" s="4" t="n">
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna (souhrn)</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>33.09</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Minerální vlna mezi krokve – Knauf Unifit 035 160 mm</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 035 160 mm</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035 160 mm</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>160 mm</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>75.53</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>242.24</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>18296</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm. Specifikace 1200×4000; DEK 1200×3200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Minerální vlna plénum – Knauf Unifit 035 140 mm (L) / full gap (R)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 035</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035 140 mm</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>L 140 / P 429 mm</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.65 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>UD 28×27</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>UD profil</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Rigips UD (obvod kastlíku)</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>28×27</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="K15" s="13" t="n">
-        <v>336</v>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
+      <c r="I15" s="9" t="n">
+        <v>23.01</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>1514.29</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>34847</v>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Levá ×140/80 vůči původním 80 mm, pravá plná mezera 429 mm. Objem modelu 20.92 m³.</t>
         </is>
       </c>
     </row>
@@ -3592,30 +3664,30 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Zavětrovací pásky 40×2</t>
+          <t>Minerální vlna kastlík + štíty</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Ocelová páska</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>Knauf Unifit 035</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Knauf Insulation Unifit 035</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>40×2</t>
+          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>32.6</v>
+        <v>5.37</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -3624,22 +3696,18 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K16" s="13" t="n">
-        <v>896</v>
-      </c>
+        <v>5.91</v>
+      </c>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>orientační ocelová páska 40×2</t>
+          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: přesný typ.</t>
+          <t>Kastlík 1.90 + štíty 3.47 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
@@ -3649,26 +3717,26 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>UD 28×27</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>Rigips UD (obvod kastlíku)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>28×27</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
-        <v>31.4</v>
+        <v>10.5</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -3677,26 +3745,26 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I17" s="6" t="n">
-        <v>33.9</v>
+        <v>11.5</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>180</v>
+        <v>29.21</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>6099</v>
+        <v>336</v>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
@@ -3706,30 +3774,30 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>17</v>
+        <v>32.6</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -3738,22 +3806,22 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>18.7</v>
+        <v>35.8</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>150</v>
+        <v>896</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
@@ -3763,26 +3831,26 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Spirála Ø160</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>VZT potrubí</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobce VZT dosud nezvolen</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ø160</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
-        <v>52.3</v>
+        <v>31.4</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -3791,26 +3859,26 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>57.5</v>
+        <v>33.9</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>3164</v>
+        <v>6099</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační spirála Ø160 pozink</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>3 trasy v kastlíku.</t>
         </is>
       </c>
     </row>
@@ -3820,117 +3888,231 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K21" s="13" t="n">
+        <v>3164</v>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F22" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I22" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J20" s="12" t="n">
+      <c r="J22" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K20" s="13" t="n">
+      <c r="K22" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="15" t="n"/>
-      <c r="H22" s="15" t="n"/>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="16" t="n">
-        <v>100949</v>
-      </c>
-      <c r="L22" s="15" t="n"/>
-      <c r="M22" s="15" t="n"/>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna (souhrn)</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
-      <c r="J23" s="18" t="n"/>
-      <c r="K23" s="18" t="n"/>
-      <c r="L23" s="18" t="n"/>
-      <c r="M23" s="18" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="16" t="n">
+        <v>153876</v>
+      </c>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna kastlík + štíty</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="18" t="n"/>
+      <c r="J25" s="18" t="n"/>
+      <c r="K25" s="18" t="n"/>
+      <c r="L25" s="18" t="n"/>
+      <c r="M25" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A25:M25"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A24:J24"/>
     <mergeCell ref="A23:M23"/>
   </mergeCells>
   <hyperlinks>
@@ -3945,6 +4127,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4103,7 +4288,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>12.13 m²</t>
+          <t>11.31 m²</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4300,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>8.74 m²</t>
+          <t>8.32 m²</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Obývák: 60/100 mm NaturHeld and a 40° UD joint at the soffit
The ceiling now follows the soffit CD. Wool below the rafters is whatever depth remains, and the product stays undecided.

Co-authored-by: Petr Sima <ptea.sima@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -736,60 +736,56 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="7" t="n">
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Akustická deska</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska ρ 140</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140, tl. 80 mm (P+D 1880×615)</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>80 mm</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140, 60 mm levá / 100 mm pravá</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>60 / 100 mm</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>71</v>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="6" t="n">
         <v>79.52</v>
       </c>
-      <c r="J5" s="10" t="n">
-        <v>534</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>42464</v>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1880-615-mm-tl-80-mm-pero-drazka-15725.html</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>Šroubováno přes GKF do CD @ 625 mm. Bez Flex / bez latí na šikmině.</t>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Levá 35.50 m² × 60 mm, pravá 35.50 m² × 100 mm. Šroubováno přes GKF do CD @ 625 mm. Cenu 60 a 100 mm ověřit (80 mm už neplatí).</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1013,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Kotvení z boku krokve. Modelové svěšení 139 mm, noha 200 mm.</t>
+          <t>Kotvení z boku krokve. Modelové svěšení 73 mm, noha 200 mm.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1070,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina. Nejdelší svěšení v modelu 428 mm (u okapu).</t>
+          <t>Pravá šikmina. Nejdelší svěšení v modelu 322 mm (u okapu).</t>
         </is>
       </c>
     </row>
@@ -1089,12 +1085,12 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035, 160 mm</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1118,15 +1114,11 @@
       <c r="I11" s="9" t="n">
         <v>75.53</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>242.24</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>18296</v>
-      </c>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -1148,21 +1140,21 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035 140 mm (L) / plná mezera (P)</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>L 140 mm / P 429 mm</t>
+          <t>L 74 mm / P 323 mm</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>20.92</v>
+        <v>14.74</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -1175,22 +1167,18 @@
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>23.01</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>1514.29</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>34847</v>
-      </c>
+        <v>16.21</v>
+      </c>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Levá 140 mm. Pravá plná mezera 429 mm (140+140+150 nebo 200+220), bez vzduchu. Objem z modelu 20.92 m³ (celá vlna šikmin 31.84 − pole 10.92). Specifikace uvádí roli 140 mm 1200×4500; DEK aktuálně 1200×3700 (4,44 m²).</t>
+          <t>Levá 73.7 mm, pravá 323.0 mm nad GKF, pod krokvemi. Objem z modelu 14.74 m³ (celá vlna šikmin 25.65 − pole 10.92).</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1319,7 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
       <c r="K16" s="16" t="n">
-        <v>114673</v>
+        <v>19065</v>
       </c>
       <c r="L16" s="15" t="n"/>
       <c r="M16" s="15" t="n"/>
@@ -1339,7 +1327,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Krov (nosná konstrukce)</t>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Akustická deska; Minerální vlna mezi krokve; Minerální vlna plénum; Krov (nosná konstrukce)</t>
         </is>
       </c>
       <c r="B17" s="18" t="n"/>
@@ -1371,8 +1359,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1513,7 +1499,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>33.92</v>
+        <v>38.27</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1526,7 +1512,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>37.31</v>
+        <v>42.1</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -1537,7 +1523,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>11.31 m² × 3,0 = 33.9 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
+          <t>12.76 m² × 3,0 = 38.3 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1552,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>28.27</v>
+        <v>31.89</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1579,7 +1565,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>31.09</v>
+        <v>35.08</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -1590,7 +1576,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>11.31 m² × 2,5 = 28.3 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
+          <t>12.76 m² × 2,5 = 31.9 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1605,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>11.31</v>
+        <v>12.76</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1632,13 +1618,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>12.66</v>
+        <v>14.29</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3368</v>
+        <v>3801</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -1676,7 +1662,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.9</v>
+        <v>1.78</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1689,13 +1675,13 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>2.09</v>
+        <v>1.95</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -1757,7 +1743,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
+          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 52.29 bm (5 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1772,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>6.76</v>
+        <v>4.98</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1799,13 +1785,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>7.57</v>
+        <v>5.58</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>877</v>
+        <v>646</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -2014,7 +2000,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>31.4</v>
+        <v>10.5</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -2027,13 +2013,13 @@
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>34.5</v>
+        <v>11.5</v>
       </c>
       <c r="J12" s="12" t="n">
         <v>55</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>1898</v>
+        <v>633</v>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
@@ -2128,7 +2114,7 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>20.9</v>
+        <v>10.5</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -2141,13 +2127,13 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>23</v>
+        <v>11.5</v>
       </c>
       <c r="J14" s="12" t="n">
         <v>55</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>1265</v>
+        <v>633</v>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
@@ -2248,7 +2234,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16345</v>
+        <v>14648</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2430,7 +2416,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>17.18</v>
+        <v>18.19</v>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
@@ -2443,13 +2429,13 @@
         </is>
       </c>
       <c r="I3" s="9" t="n">
-        <v>19.24</v>
+        <v>20.37</v>
       </c>
       <c r="J3" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>1847</v>
+        <v>1956</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
@@ -2489,7 +2475,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>98.40000000000001</v>
+        <v>103.2</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2502,13 +2488,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>108.2</v>
+        <v>113.5</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3160</v>
+        <v>3315</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2548,7 +2534,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2561,13 +2547,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>36.7</v>
+        <v>37.8</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>17515</v>
+        <v>18031</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2658,7 +2644,7 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -2671,13 +2657,13 @@
         </is>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1.19</v>
+        <v>1.28</v>
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -2713,7 +2699,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2.5</v>
+        <v>2.68</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -2726,13 +2712,13 @@
         </is>
       </c>
       <c r="I8" s="6" t="n">
-        <v>2.75</v>
+        <v>2.94</v>
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -2772,7 +2758,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>22523</v>
+        <v>23301</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -2821,7 +2807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2950,7 +2936,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>246.92</v>
+        <v>251.28</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -2963,7 +2949,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>271.61</v>
+        <v>276.4</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -2974,7 +2960,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Šikminy+kastlík 82.31 m² → 246.9 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
+          <t>Šikminy+kastlík 83.76 m² → 251.3 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +2989,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>205.77</v>
+        <v>209.4</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -3016,7 +3002,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>226.35</v>
+        <v>230.34</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -3027,150 +3013,144 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>205.8 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="7" t="n">
+          <t>209.4 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 — 80 mm</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 — 60 mm levá</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 / 80 mm</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>80 mm</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>71</v>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 / 60 mm</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>60 mm</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I5" s="9" t="n">
-        <v>79.52</v>
-      </c>
-      <c r="J5" s="10" t="n">
-        <v>534</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>42464</v>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1880-615-mm-tl-80-mm-pero-drazka-15725.html</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>Šikminy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 — 40 mm</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="I5" s="6" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Okenní šikmina. Cenu ověřit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 — 100 mm pravá</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 / 40 mm</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>40 mm</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>11.31</v>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 / 100 mm</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>100 mm</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I6" s="9" t="n">
-        <v>12.66</v>
-      </c>
-      <c r="J6" s="10" t="n">
-        <v>266</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>3368</v>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1250-600-mm-tl-40-mm-15722.html</t>
-        </is>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>Kastlík.</t>
+      <c r="I6" s="6" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Šikmina u skříní. Cenu ověřit.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Parozábrana</t>
+          <t>NaturHeld 140 — 40 mm</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Jutafol N AL 170 Speciál</t>
+          <t>Dřevovláknitá deska</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Jutafol N AL 170 Speciál</t>
+          <t>NaturHeld 140 / 40 mm</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>role 75 m²</t>
+          <t>40 mm</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>71</v>
+        <v>12.76</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -3179,55 +3159,55 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>78.09999999999999</v>
+        <v>14.29</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>35.73</v>
+        <v>266</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2791</v>
+        <v>3801</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
+          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1250-600-mm-tl-40-mm-15722.html</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
+          <t>Kastlík.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton RF 12,5</t>
+          <t>Parozábrana</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>GKF/RF</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Rigips RF 12,5</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>12,5 mm</t>
+          <t>role 75 m²</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>77.76000000000001</v>
+        <v>71</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3236,46 +3216,46 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>12 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>87.09</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>115.88</v>
+        <v>35.73</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>10092</v>
+        <v>2791</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Šikminy + víko kastlíku.</t>
+          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
+          <t>Sádrokarton RF 12,5</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>GKB plná</t>
+          <t>GKF/RF</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Rigips RB/RF 12,5</t>
+          <t>Rigips RF 12,5</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3284,7 +3264,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>17.18</v>
+        <v>75.98</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -3297,165 +3277,165 @@
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>19.24</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>96</v>
+        <v>115.88</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1847</v>
+        <v>9861</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
+          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Šikminy + víko kastlíku.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Profil R-CD 60×27</t>
+          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>CD profil</t>
+          <t>GKB plná</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips R-CD</t>
+          <t>Rigips RB/RF 12,5</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>60×27</t>
+          <t>12,5 mm</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>227.1</v>
+        <v>18.19</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>249.8</v>
+        <v>20.37</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>29.21</v>
+        <v>96</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7297</v>
+        <v>1956</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Šikminy + kastlík + štíty.</t>
+          <t>Štíty.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm DK Mont</t>
+          <t>Profil R-CD 60×27</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm</t>
+          <t>CD profil</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>DK Mont 3631100170</t>
+          <t>Rigips R-CD</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>200 mm</t>
+          <t>60×27</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>52</v>
+        <v>231.9</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>56.2</v>
+        <v>255.1</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>12.52</v>
+        <v>29.21</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>703</v>
+        <v>7452</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Okenní šikmina. Svěšení 139 mm. Balení 100 ks.</t>
+          <t>Šikminy + kastlík + štíty.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Nonius sada</t>
+          <t>Přímý závěs 200 mm DK Mont</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>H+S+2× závlačka</t>
+          <t>Přímý závěs 200 mm</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
+          <t>DK Mont 3631100170</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>200 mm</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -3468,51 +3448,51 @@
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>84.2</v>
+        <v>56.2</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>32.07</v>
+        <v>12.52</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>2702</v>
+        <v>703</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina + kastlík. Svěšení šikminy 428 mm, kastlík 406 mm.</t>
+          <t>Okenní šikmina. Svěšení 73 mm. Balení 100 ks.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Akustický třmen KB517112</t>
+          <t>Nonius sada</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Třmen + Sylomer</t>
+          <t>H+S+2× závlačka</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Rigips KB517112</t>
+          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>440</t>
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3525,165 +3505,161 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>36.7</v>
+        <v>84.2</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>477</v>
+        <v>32.07</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>17515</v>
+        <v>2702</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Pravá šikmina + kastlík. Svěšení šikminy 322 mm, kastlík 406 mm.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Akustický třmen KB517112</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Třmen + Sylomer</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Rigips KB517112</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>477</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>18031</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>Štíty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Minerální vlna mezi krokve – Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Minerální vlna mezi krokve</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>160 mm</t>
         </is>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F15" s="6" t="n">
         <v>68.66</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I15" s="6" t="n">
         <v>75.53</v>
       </c>
-      <c r="J14" s="10" t="n">
-        <v>242.24</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>18296</v>
-      </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
-        </is>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm. Specifikace 1200×4000; DEK 1200×3200.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Minerální vlna plénum – Knauf Unifit 035 140 mm (L) / full gap (R)</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Knauf Unifit 035</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035 140 mm</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>L 140 / P 429 mm</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>20.92</v>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>23.01</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>1514.29</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>34847</v>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>Levá ×140/80 vůči původním 80 mm, pravá plná mezera 429 mm. Objem modelu 20.92 m³.</t>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Minerální vlna kastlík + štíty</t>
+          <t>Minerální vlna pod krokvemi</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
+          <t>L 74 / P 323 mm</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>5.37</v>
+        <v>14.74</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -3696,28 +3672,30 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>5.91</v>
+        <v>16.21</v>
       </c>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Kastlík 1.90 + štíty 3.47 m³. Tloušťky beze změny, stejný výrobek.</t>
+          <t>Nad GKF. Levá 73.7 mm, pravá 323.0 mm. Objem modelu 14.74 m³.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="4" t="n">
-        <v>15</v>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>13b</t>
+        </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>UD 28×27</t>
+          <t>UD 40° na spoji šikminy</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -3727,12 +3705,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Rigips UD (obvod kastlíku)</t>
+          <t>UD 28×27 naříznutý a ohnutý na 40°</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>28×27</t>
+          <t>40°</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
@@ -3751,53 +3729,49 @@
       <c r="I17" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="J17" s="12" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="K17" s="13" t="n">
-        <v>336</v>
-      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
+          <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. Spára akryl + páska 10.46 bm.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Zavětrovací pásky 40×2</t>
+          <t>Minerální vlna kastlík + štíty</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Ocelová páska</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>40×2</t>
+          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>32.6</v>
+        <v>5.5</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -3806,51 +3780,47 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K18" s="13" t="n">
-        <v>896</v>
-      </c>
+        <v>6.05</v>
+      </c>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>orientační ocelová páska 40×2</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: přesný typ.</t>
+          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>UD 28×27</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>Rigips UD (obvod kastlíku)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>28×27</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
-        <v>31.4</v>
+        <v>52.3</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -3859,59 +3829,59 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>33.9</v>
+        <v>57.5</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>180</v>
+        <v>29.21</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>6099</v>
+        <v>1680</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>17</v>
+        <v>32.6</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -3920,51 +3890,51 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>18.7</v>
+        <v>35.8</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>150</v>
+        <v>896</v>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Spirála Ø160</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>VZT potrubí</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobce VZT dosud nezvolen</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ø160</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>52.3</v>
+        <v>31.4</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -3973,147 +3943,261 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="I21" s="6" t="n">
-        <v>57.5</v>
+        <v>33.9</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>3164</v>
+        <v>6099</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační spirála Ø160 pozink</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>3 trasy v kastlíku.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K23" s="13" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F24" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I24" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J24" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K22" s="13" t="n">
+      <c r="K24" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="16" t="n">
-        <v>153876</v>
-      </c>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18" t="n"/>
-      <c r="K25" s="18" t="n"/>
-      <c r="L25" s="18" t="n"/>
-      <c r="M25" s="18" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="16" t="n">
+        <v>58695</v>
+      </c>
+      <c r="L26" s="15" t="n"/>
+      <c r="M26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; Minerální vlna mezi krokve; Minerální vlna pod krokvemi; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A27:M27"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A26:J26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -4128,8 +4212,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4288,7 +4370,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>11.31 m²</t>
+          <t>12.76 m²</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4382,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>8.32 m²</t>
+          <t>8.92 m²</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Living room: confirm slope wool (Unifit 033 left, NatuRoll 039 right) and price it
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -998,13 +998,13 @@
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>56.2</v>
+        <v>70.2</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>12.52</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>703</v>
+        <v>879</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -1055,13 +1055,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>70.2</v>
+        <v>56.2</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>32.07</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>2251</v>
+        <v>1801</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -1080,26 +1080,26 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Minerální vlna mezi krokve</t>
+          <t>Wool between rafters, left</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
+          <t>Glass wool, λ 0.033</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 033 160 mm</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>160 mm · řez ~790 mm</t>
+          <t>160 mm · roll 1200×2800 (3.36 m²)</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>68.66</v>
+        <v>34.33</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -1108,22 +1108,26 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>5 %</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>75.53</v>
-      </c>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
+        <v>36.05</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>278.27</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>10031</v>
+      </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+          <t>NonstopStavebniny, 935 Kč / 3.36 m² roll incl. VAT · https://www.nonstopstavebniny.cz/vata-knauf-unifit-033-tl--160-mm-tepelna-izolace-baleni-3-36-m2/</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Plocha sklonu nad místností 77.52 m² × (775/875). Šikmina po nábytek by byla 62.89 m²; model vyplňuje pole i nad kastlíkem. Specifikace uvádí roli 1200×4000; DEK aktuálně 1200×3200 (3,84 m²).</t>
+          <t>Left slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 11 rolls.</t>
         </is>
       </c>
     </row>
@@ -1135,220 +1139,342 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Minerální vlna plénum</t>
+          <t>Wool below rafters, left</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
+          <t>Glass wool, λ 0.033</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 033 80 mm</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>L 74 mm / P 323 mm</t>
+          <t>80 mm · roll 6.6 m²</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>14.74</v>
+        <v>35.5</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>215.25</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>8024</v>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Stav-Invest, 1,420.65 Kč / 6.6 m² roll incl. VAT · https://eshop.stavinvest.cz/tepelna-izolace-knauf-unifit-033-80-mm/</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>Left slope face 35.50 m², 1 layer → 6 rolls. Model cavity 73.7 mm; 80 mm fills it with light compression. U ≈ 0.121, foil 13.2 °C at −15 °C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>9c</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Wool between rafters, right</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.039</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Knauf NatuRoll Pro 039 160 mm</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>160 mm · roll 1200×4800 (5.76 m²)</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>141.49</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>Right slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 7 rolls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>9d</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Wool below rafters, right</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.039</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Knauf NatuRoll Pro 039 160 mm</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>2 × 160 = 320 mm</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>141.49</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>10548</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 323.0 mm. U ≈ 0.068, foil ≈ 14.2 °C at −15 °C; whole roof U ≈ 0.095.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Zavětrování</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Ocelová páska</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Výrobek dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>40×2 mm @ 45°</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I12" s="9" t="n">
-        <v>16.21</v>
-      </c>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>Levá 73.7 mm, pravá 323.0 mm nad GKF, pod krokvemi. Objem z modelu 14.74 m³ (celá vlna šikmin 25.65 − pole 10.92).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="52" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Zavětrování</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Ocelová páska</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>40×2 mm @ 45°</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n">
+      <c r="I15" s="6" t="n">
         <v>35.8</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="J15" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="K13" s="13" t="n">
+      <c r="K15" s="13" t="n">
         <v>896</v>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Typ pásky / kotevní prvky ještě sjednotit.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
-      <c r="A14" s="7" t="n">
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Krov (nosná konstrukce)</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Krokve</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Stávající krov</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>100/160 @ 875</t>
         </is>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F16" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n">
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>Není položka nákupu akustiky.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="15" t="n"/>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="16" t="n">
-        <v>19065</v>
-      </c>
-      <c r="L16" s="15" t="n"/>
-      <c r="M16" s="15" t="n"/>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Akustická deska; Minerální vlna mezi krokve; Minerální vlna plénum; Krov (nosná konstrukce)</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n"/>
-      <c r="J17" s="18" t="n"/>
-      <c r="K17" s="18" t="n"/>
-      <c r="L17" s="18" t="n"/>
-      <c r="M17" s="18" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="16" t="n">
+        <v>52494</v>
+      </c>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Akustická deska; Krov (nosná konstrukce)</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="18" t="n"/>
+      <c r="M19" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A19:M19"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A15:M15"/>
-    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A18:J18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -1359,6 +1485,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1681,7 +1811,7 @@
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -1743,7 +1873,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 52.29 bm (5 ks). Žádné latě, žádné podložky.</t>
+          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 20.92 bm (2 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2793,7 @@
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -2718,7 +2848,7 @@
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -2807,7 +2937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3435,7 +3565,7 @@
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -3448,13 +3578,13 @@
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>56.2</v>
+        <v>70.2</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>12.52</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>703</v>
+        <v>879</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
@@ -3492,7 +3622,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3505,13 +3635,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>84.2</v>
+        <v>70.2</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>32.07</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>2702</v>
+        <v>2251</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3581,307 +3711,325 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="4" t="n">
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna mezi krokve</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>160 mm</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>68.66</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Wool between rafters, left</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.033</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 033 160 mm</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>160 mm · roll 1200×2800 (3.36 m²)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>278.27</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>10031</v>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 935 Kč / 3.36 m² roll incl. VAT · https://www.nonstopstavebniny.cz/vata-knauf-unifit-033-tl--160-mm-tepelna-izolace-baleni-3-36-m2/</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Left slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 11 rolls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>12b</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Wool below rafters, left</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.033</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Knauf Unifit 033 80 mm</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>80 mm · roll 6.6 m²</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>215.25</v>
+      </c>
+      <c r="K16" s="11" t="n">
+        <v>8024</v>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Stav-Invest, 1,420.65 Kč / 6.6 m² roll incl. VAT · https://eshop.stavinvest.cz/tepelna-izolace-knauf-unifit-033-80-mm/</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>Left slope face 35.50 m², 1 layer → 6 rolls. Model cavity 73.7 mm; 80 mm fills it with light compression. U ≈ 0.121, foil 13.2 °C at −15 °C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>12c</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Wool between rafters, right</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.039</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Knauf NatuRoll Pro 039 160 mm</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>160 mm · roll 1200×4800 (5.76 m²)</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>141.49</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>Right slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 7 rolls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Wool below rafters, right</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.039</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Knauf NatuRoll Pro 039 160 mm</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2 × 160 = 320 mm</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>141.49</v>
+      </c>
+      <c r="K18" s="11" t="n">
+        <v>10548</v>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 323.0 mm. U ≈ 0.068, foil ≈ 14.2 °C at −15 °C; whole roof U ≈ 0.095.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>13b</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>UD 40° na spoji šikminy</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>UD profil</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>UD 28×27 naříznutý a ohnutý na 40°</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>40°</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n">
-        <v>75.53</v>
-      </c>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="52" customHeight="1">
-      <c r="A16" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna pod krokvemi</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>L 74 / P 323 mm</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>14.74</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="n">
-        <v>16.21</v>
-      </c>
-      <c r="J16" s="6" t="n"/>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
-        </is>
-      </c>
-      <c r="M16" s="4" t="inlineStr">
-        <is>
-          <t>Nad GKF. Levá 73.7 mm, pravá 323.0 mm. Objem modelu 14.74 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>13b</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>UD 40° na spoji šikminy</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>UD profil</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>UD 28×27 naříznutý a ohnutý na 40°</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>40°</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="n">
+      <c r="I19" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. Spára akryl + páska 10.46 bm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="A18" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="n">
-        <v>6.05</v>
-      </c>
-      <c r="J18" s="6" t="n"/>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
-        </is>
-      </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>UD 28×27</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>UD profil</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Rigips UD (obvod kastlíku)</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>28×27</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>52.3</v>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="K19" s="13" t="n">
-        <v>1680</v>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Zavětrovací pásky 40×2</t>
+          <t>Minerální vlna kastlík + štíty</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Ocelová páska</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>40×2</t>
+          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>32.6</v>
+        <v>5.5</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -3890,51 +4038,47 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J20" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K20" s="13" t="n">
-        <v>896</v>
-      </c>
+        <v>6.05</v>
+      </c>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>orientační ocelová páska 40×2</t>
+          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: přesný typ.</t>
+          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>UD 28×27</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>Rigips UD (obvod kastlíku)</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>28×27</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>31.4</v>
+        <v>20.9</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -3943,59 +4087,59 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I21" s="6" t="n">
-        <v>33.9</v>
+        <v>23</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>180</v>
+        <v>29.21</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>6099</v>
+        <v>672</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>17</v>
+        <v>32.6</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -4004,51 +4148,51 @@
         </is>
       </c>
       <c r="I22" s="6" t="n">
-        <v>18.7</v>
+        <v>35.8</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="K22" s="13" t="n">
-        <v>150</v>
+        <v>896</v>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Spirála Ø160</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>VZT potrubí</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobce VZT dosud nezvolen</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ø160</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>20.9</v>
+        <v>31.4</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -4057,147 +4201,261 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="I23" s="6" t="n">
-        <v>23</v>
+        <v>33.9</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="K23" s="13" t="n">
-        <v>1265</v>
+        <v>6099</v>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační spirála Ø160 pozink</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>3 trasy v kastlíku.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K24" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J25" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K25" s="13" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I24" s="6" t="n">
+      <c r="I26" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J26" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K24" s="13" t="n">
+      <c r="K26" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n"/>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="15" t="n"/>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="16" t="n">
-        <v>58695</v>
-      </c>
-      <c r="L26" s="15" t="n"/>
-      <c r="M26" s="15" t="n"/>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; Minerální vlna mezi krokve; Minerální vlna pod krokvemi; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="M27" s="18" t="n"/>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="n"/>
+      <c r="K28" s="16" t="n">
+        <v>91115</v>
+      </c>
+      <c r="L28" s="15" t="n"/>
+      <c r="M28" s="15" t="n"/>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
+      <c r="L29" s="18" t="n"/>
+      <c r="M29" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A28:J28"/>
     <mergeCell ref="A27:M27"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A29:M29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -4212,6 +4470,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Living room: 2x GKF on the road-side (right) slope for road noise
Room face and ceiling height unchanged; the right CD plane moves up 12.5 mm.
Right below-rafter wool cavity 323.0 -> 310.5 mm (2x160 NatuRoll ~3 % compressed).
Ridge: GKF room faces still meet 31 mm right of the false ridge; the outer layer
is bevelled to the CD meeting line 41 mm right of it. Soffit UD bend sits 16 mm
up the soffit CD cheek. BOM: 2nd GKF layer, TN 35 screws, Vario filler.
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -904,145 +904,147 @@
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>6</v>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Rošt CD</t>
+          <t>Podkladní deska, 2. vrstva (pravá šikmina)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Profil CD 60×27</t>
+          <t>Sádrokarton GKF / RF</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Rigips R-CD profil 27/60/27</t>
+          <t>Rigips RF (DF) 12,5 mm</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>60×27 mm @ 625 mm ⊥ krokvím</t>
+          <t>12.5 mm</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>99.90000000000001</v>
+        <v>35.5</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>109.9</v>
+        <v>39.76</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>29.21</v>
+        <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>3209</v>
+        <v>4607</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>9 profilů × 11.10 m.</t>
+          <t>Second layer on the road-side slope for road noise. Joints staggered against the first layer. Same 3 mm acrylic joint at the soffit.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Závěs — okenní šikmina</t>
+          <t>Rošt CD</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm DK Mont</t>
+          <t>Profil CD 60×27</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm DK Mont 3631100170</t>
+          <t>Rigips R-CD profil 27/60/27</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>200 mm</t>
+          <t>60×27 mm @ 625 mm ⊥ krokvím</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>65</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>70.2</v>
+        <v>109.9</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>12.52</v>
+        <v>29.21</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>879</v>
+        <v>3209</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Kotvení z boku krokve. Modelové svěšení 73 mm, noha 200 mm.</t>
+          <t>9 profilů × 11.10 m.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Závěs — šikmina u skříní</t>
+          <t>Závěs — okenní šikmina</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Nonius sada (horní+spodní+2× závlačka)</t>
+          <t>Přímý závěs 200 mm DK Mont</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius horní 440 + spodní CD + 2× závlačka</t>
+          <t>Přímý závěs 200 mm DK Mont 3631100170</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>horní 440 mm</t>
+          <t>200 mm</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -1055,169 +1057,167 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>56.2</v>
+        <v>70.2</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>32.07</v>
+        <v>12.52</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>1801</v>
+        <v>879</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina. Nejdelší svěšení v modelu 322 mm (u okapu).</t>
+          <t>Kotvení z boku krokve. Modelové svěšení 73 mm, noha 200 mm.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Závěs — šikmina u skříní</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Nonius sada (horní+spodní+2× závlačka)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Rigips Nonius horní 440 + spodní CD + 2× závlačka</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>horní 440 mm</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>32.07</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>1801</v>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>Pravá šikmina. Nejdelší svěšení v modelu 309 mm (u okapu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Wool between rafters, left</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Glass wool, λ 0.033</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Knauf Unifit 033 160 mm</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>160 mm · roll 1200×2800 (3.36 m²)</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F12" s="9" t="n">
         <v>34.33</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I12" s="9" t="n">
         <v>36.05</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="J12" s="10" t="n">
         <v>278.27</v>
       </c>
-      <c r="K11" s="11" t="n">
+      <c r="K12" s="11" t="n">
         <v>10031</v>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>NonstopStavebniny, 935 Kč / 3.36 m² roll incl. VAT · https://www.nonstopstavebniny.cz/vata-knauf-unifit-033-tl--160-mm-tepelna-izolace-baleni-3-36-m2/</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Left slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 11 rolls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>9b</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Wool below rafters, left</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Glass wool, λ 0.033</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Unifit 033 80 mm</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>80 mm · roll 6.6 m²</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>5 %</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>37.28</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>215.25</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>8024</v>
-      </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>Stav-Invest, 1,420.65 Kč / 6.6 m² roll incl. VAT · https://eshop.stavinvest.cz/tepelna-izolace-knauf-unifit-033-80-mm/</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>Left slope face 35.50 m², 1 layer → 6 rolls. Model cavity 73.7 mm; 80 mm fills it with light compression. U ≈ 0.121, foil 13.2 °C at −15 °C.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>9c</t>
+          <t>9b</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Wool between rafters, right</t>
+          <t>Wool below rafters, left</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Glass wool, λ 0.039</t>
+          <t>Glass wool, λ 0.033</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Knauf NatuRoll Pro 039 160 mm</t>
+          <t>Knauf Unifit 033 80 mm</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>160 mm · roll 1200×4800 (5.76 m²)</t>
+          <t>80 mm · roll 6.6 m²</t>
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>34.33</v>
+        <v>35.5</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -1230,34 +1230,34 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>36.05</v>
+        <v>37.28</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>141.49</v>
+        <v>215.25</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>5100</v>
+        <v>8024</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+          <t>Stav-Invest, 1,420.65 Kč / 6.6 m² roll incl. VAT · https://eshop.stavinvest.cz/tepelna-izolace-knauf-unifit-033-80-mm/</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Right slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 7 rolls.</t>
+          <t>Left slope face 35.50 m², 1 layer → 6 rolls. Model cavity 73.7 mm; 80 mm fills it with light compression. U ≈ 0.121, foil 13.2 °C at −15 °C.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>9d</t>
+          <t>9c</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Wool below rafters, right</t>
+          <t>Wool between rafters, right</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>2 × 160 = 320 mm</t>
+          <t>160 mm · roll 1200×4800 (5.76 m²)</t>
         </is>
       </c>
       <c r="F14" s="9" t="n">
-        <v>71</v>
+        <v>34.33</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
@@ -1289,192 +1289,251 @@
         </is>
       </c>
       <c r="I14" s="9" t="n">
-        <v>74.55</v>
+        <v>36.05</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>141.49</v>
       </c>
       <c r="K14" s="11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>Right slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 7 rolls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>9d</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Wool below rafters, right</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Glass wool, λ 0.039</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Knauf NatuRoll Pro 039 160 mm</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>2 × 160 = 320 mm</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>141.49</v>
+      </c>
+      <c r="K15" s="11" t="n">
         <v>10548</v>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 323.0 mm. U ≈ 0.068, foil ≈ 14.2 °C at −15 °C; whole roof U ≈ 0.095.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 310.5 mm (2× GKF on this side), so 2 × 160 is compressed ~3 %. U ≈ 0.070, foil ≈ 13.9 °C at −15 °C; whole roof U ≈ 0.096.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Zavětrování</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Ocelová páska</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>40×2 mm @ 45°</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F16" s="6" t="n">
         <v>32.6</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I16" s="6" t="n">
         <v>35.8</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J16" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="K15" s="13" t="n">
+      <c r="K16" s="13" t="n">
         <v>896</v>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Typ pásky / kotevní prvky ještě sjednotit.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" s="7" t="n">
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Krov (nosná konstrukce)</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Krokve</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Stávající krov</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>100/160 @ 875</t>
         </is>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F17" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="n">
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="9" t="n"/>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Není položka nákupu akustiky.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="15" t="n"/>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="16" t="n">
-        <v>52494</v>
-      </c>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="16" t="n">
+        <v>57101</v>
+      </c>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Akustická deska; Krov (nosná konstrukce)</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
-      <c r="H19" s="18" t="n"/>
-      <c r="I19" s="18" t="n"/>
-      <c r="J19" s="18" t="n"/>
-      <c r="K19" s="18" t="n"/>
-      <c r="L19" s="18" t="n"/>
-      <c r="M19" s="18" t="n"/>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="18" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="18" t="n"/>
+      <c r="H20" s="18" t="n"/>
+      <c r="I20" s="18" t="n"/>
+      <c r="J20" s="18" t="n"/>
+      <c r="K20" s="18" t="n"/>
+      <c r="L20" s="18" t="n"/>
+      <c r="M20" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A20:M20"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A18:M18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -1489,6 +1548,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2937,7 +2997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3427,22 +3487,24 @@
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="7" t="n">
-        <v>7</v>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>6b</t>
+        </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
+          <t>GKF RF 12.5, 2nd layer, right slope</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>GKB plná</t>
+          <t>GKF/RF</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips RB/RF 12,5</t>
+          <t>Rigips RF 12,5</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3451,7 +3513,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>18.19</v>
+        <v>35.5</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3464,55 +3526,57 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>20.37</v>
+        <v>39.76</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>96</v>
+        <v>115.88</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>1956</v>
+        <v>4607</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
+          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Road-side slope only (2× GKF for road noise). 35.50 m² → 16 boards 1250×2000.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>8</v>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6c</t>
+        </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Profil R-CD 60×27</t>
+          <t>Screws TN 35, 2nd GKF layer</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>CD profil</t>
+          <t>Drywall screw</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Rigips R-CD</t>
+          <t>DK Mont TN 35</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>60×27</t>
+          <t>3.5×35</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>231.9</v>
+        <v>355</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -3521,739 +3585,741 @@
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>255.1</v>
+        <v>390.5</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>29.21</v>
+        <v>0.22</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>7452</v>
+        <v>86</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>DEK DK Mont TN 35, 220.78 Kč / 1000 pcs incl. VAT · https://www.dek.cz/produkty/detail/3631100059-rychlosroub-tn-35-profi-1000ks-bal-dkm</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Šikminy + kastlík + štíty.</t>
+          <t>Outer layer @ ≤170 mm on CD @ 625 mm ≈ 10 pcs/m². First layer keeps TN 25 at wider spacing (not priced, as before).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="7" t="n">
-        <v>9</v>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>6d</t>
+        </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm DK Mont</t>
+          <t>Joint compound, 1st-layer joints</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm</t>
+          <t>Gypsum filler</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>DK Mont 3631100170</t>
+          <t>Rigips Vario 25 kg</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>200 mm</t>
+          <t>25 kg</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>65</v>
+        <v>10.65</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>70.2</v>
+        <v>11.72</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>12.52</v>
+        <v>39.32</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>879</v>
+        <v>461</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
+          <t>izosystems.cz Rigips Vario, 983 Kč / 25 kg incl. VAT · https://izosystems.cz/stavebni-chemie/1000-sadrovy-tmel-rigips-vario-25-kg.html</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Okenní šikmina. Svěšení 73 mm. Balení 100 ks.</t>
+          <t>Inner-layer joints filled (no tape) at 0.3 kg/m². Outer-layer joints and tape as for the single board (not priced, as before).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Nonius sada</t>
+          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>H+S+2× závlačka</t>
+          <t>GKB plná</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
+          <t>Rigips RB/RF 12,5</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>12,5 mm</t>
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>65</v>
+        <v>18.19</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>70.2</v>
+        <v>20.37</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>32.07</v>
+        <v>96</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>2251</v>
+        <v>1956</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina + kastlík. Svěšení šikminy 322 mm, kastlík 406 mm.</t>
+          <t>Štíty.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Akustický třmen KB517112</t>
+          <t>Profil R-CD 60×27</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Třmen + Sylomer</t>
+          <t>CD profil</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Rigips KB517112</t>
+          <t>Rigips R-CD</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>60×27</t>
         </is>
       </c>
       <c r="F14" s="9" t="n">
-        <v>35</v>
+        <v>231.9</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I14" s="9" t="n">
-        <v>37.8</v>
+        <v>255.1</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>477</v>
+        <v>29.21</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>18031</v>
+        <v>7452</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Šikminy + kastlík + štíty.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Přímý závěs 200 mm DK Mont</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Přímý závěs 200 mm</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>DK Mont 3631100170</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>200 mm</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>12.52</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>879</v>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Okenní šikmina. Svěšení 73 mm. Balení 100 ks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Nonius sada</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>H+S+2× závlačka</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>440</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>32.07</v>
+      </c>
+      <c r="K16" s="11" t="n">
+        <v>2251</v>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>Pravá šikmina + kastlík. Svěšení šikminy 309 mm, kastlík 406 mm. Load with 2× GKF ≈ 22 kg per hanger point (was ≈ 17 kg); Nonius load class 0.40 kN, so OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Akustický třmen KB517112</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Třmen + Sylomer</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Rigips KB517112</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>477</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>18031</v>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>Štíty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Wool between rafters, left</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Glass wool, λ 0.033</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Knauf Unifit 033 160 mm</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>160 mm · roll 1200×2800 (3.36 m²)</t>
         </is>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F18" s="9" t="n">
         <v>34.33</v>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
+      <c r="I18" s="9" t="n">
         <v>36.05</v>
       </c>
-      <c r="J15" s="10" t="n">
+      <c r="J18" s="10" t="n">
         <v>278.27</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K18" s="11" t="n">
         <v>10031</v>
       </c>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>NonstopStavebniny, 935 Kč / 3.36 m² roll incl. VAT · https://www.nonstopstavebniny.cz/vata-knauf-unifit-033-tl--160-mm-tepelna-izolace-baleni-3-36-m2/</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
         <is>
           <t>Left slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 11 rolls.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>12b</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Wool below rafters, left</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Glass wool, λ 0.033</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Knauf Unifit 033 80 mm</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>80 mm · roll 6.6 m²</t>
         </is>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F19" s="9" t="n">
         <v>35.5</v>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="I19" s="9" t="n">
         <v>37.28</v>
       </c>
-      <c r="J16" s="10" t="n">
+      <c r="J19" s="10" t="n">
         <v>215.25</v>
       </c>
-      <c r="K16" s="11" t="n">
+      <c r="K19" s="11" t="n">
         <v>8024</v>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>Stav-Invest, 1,420.65 Kč / 6.6 m² roll incl. VAT · https://eshop.stavinvest.cz/tepelna-izolace-knauf-unifit-033-80-mm/</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>Left slope face 35.50 m², 1 layer → 6 rolls. Model cavity 73.7 mm; 80 mm fills it with light compression. U ≈ 0.121, foil 13.2 °C at −15 °C.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>12c</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Wool between rafters, right</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Glass wool, λ 0.039</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Knauf NatuRoll Pro 039 160 mm</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>160 mm · roll 1200×4800 (5.76 m²)</t>
         </is>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F20" s="9" t="n">
         <v>34.33</v>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="I17" s="9" t="n">
+      <c r="I20" s="9" t="n">
         <v>36.05</v>
       </c>
-      <c r="J17" s="10" t="n">
+      <c r="J20" s="10" t="n">
         <v>141.49</v>
       </c>
-      <c r="K17" s="11" t="n">
+      <c r="K20" s="11" t="n">
         <v>5100</v>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L20" s="7" t="inlineStr">
         <is>
           <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="M20" s="7" t="inlineStr">
         <is>
           <t>Right slope 38.76 m² × (775/875) net of rafters = 34.33 m² → 7 rolls.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="44" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>12d</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Wool below rafters, right</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Glass wool, λ 0.039</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Knauf NatuRoll Pro 039 160 mm</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>2 × 160 = 320 mm</t>
         </is>
       </c>
-      <c r="F18" s="9" t="n">
+      <c r="F21" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="I18" s="9" t="n">
+      <c r="I21" s="9" t="n">
         <v>74.55</v>
       </c>
-      <c r="J18" s="10" t="n">
+      <c r="J21" s="10" t="n">
         <v>141.49</v>
       </c>
-      <c r="K18" s="11" t="n">
+      <c r="K21" s="11" t="n">
         <v>10548</v>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L21" s="7" t="inlineStr">
         <is>
           <t>NonstopStavebniny, 815 Kč / 5.76 m² roll incl. VAT · https://www.nonstopstavebniny.cz/mineralni-vata-knauf-naturoll-pro-039-tepelna-izolace-160-mm-2/</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 323.0 mm. U ≈ 0.068, foil ≈ 14.2 °C at −15 °C; whole roof U ≈ 0.095.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>Right slope face 35.50 m² × 2 layers = 71.00 m² → 13 rolls. Model cavity 310.5 mm (2× GKF on this side), so 2 × 160 is compressed ~3 %. U ≈ 0.070, foil ≈ 13.9 °C at −15 °C; whole roof U ≈ 0.096.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>UD 40° na spoji šikminy</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>UD profil</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>UD 28×27 naříznutý a ohnutý na 40°</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>40°</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F22" s="6" t="n">
         <v>10.5</v>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I22" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. Spára akryl + páska 10.46 bm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="52" customHeight="1">
-      <c r="A20" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>zatím neurčeno</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="n">
-        <v>6.05</v>
-      </c>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>UD 28×27</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>UD profil</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Rigips UD (obvod kastlíku)</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>28×27</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="K21" s="13" t="n">
-        <v>672</v>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="inlineStr">
-        <is>
-          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="52" customHeight="1">
-      <c r="A22" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Zavětrovací pásky 40×2</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Ocelová páska</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>40×2</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K22" s="13" t="n">
-        <v>896</v>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>orientační ocelová páska 40×2</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>Minerální vlna kastlík + štíty</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>31.4</v>
+        <v>5.5</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I23" s="6" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>180</v>
-      </c>
-      <c r="K23" s="13" t="n">
-        <v>6099</v>
-      </c>
+        <v>6.05</v>
+      </c>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>Soffit and gable wool product still to confirm (slope wool is decided).</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>UD 28×27</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Rigips UD (obvod kastlíku)</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>28×27</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>17</v>
+        <v>20.9</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -4262,51 +4328,51 @@
         </is>
       </c>
       <c r="I24" s="6" t="n">
-        <v>18.7</v>
+        <v>23</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>8</v>
+        <v>29.21</v>
       </c>
       <c r="K24" s="13" t="n">
-        <v>150</v>
+        <v>672</v>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>20.9</v>
+        <v>32.6</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -4319,143 +4385,314 @@
         </is>
       </c>
       <c r="I25" s="6" t="n">
-        <v>23</v>
+        <v>35.8</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>1265</v>
+        <v>896</v>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="52" customHeight="1">
       <c r="A26" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Spirála Ø160</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>VZT potrubí</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Výrobce VZT dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Ø160</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="J26" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="K26" s="13" t="n">
+        <v>6099</v>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>orientační spirála Ø160 pozink</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>3 trasy v kastlíku.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K27" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K28" s="13" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="52" customHeight="1">
+      <c r="A29" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I26" s="6" t="n">
+      <c r="I29" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J26" s="12" t="n">
+      <c r="J29" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K26" s="13" t="n">
+      <c r="K29" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="15" t="n"/>
-      <c r="H28" s="15" t="n"/>
-      <c r="I28" s="15" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="16" t="n">
-        <v>91115</v>
-      </c>
-      <c r="L28" s="15" t="n"/>
-      <c r="M28" s="15" t="n"/>
-    </row>
-    <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="15" t="n"/>
+      <c r="I31" s="15" t="n"/>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="16" t="n">
+        <v>96269</v>
+      </c>
+      <c r="L31" s="15" t="n"/>
+      <c r="M31" s="15" t="n"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
         </is>
       </c>
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="18" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="18" t="n"/>
-      <c r="I29" s="18" t="n"/>
-      <c r="J29" s="18" t="n"/>
-      <c r="K29" s="18" t="n"/>
-      <c r="L29" s="18" t="n"/>
-      <c r="M29" s="18" t="n"/>
+      <c r="B32" s="18" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="18" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="18" t="n"/>
+      <c r="J32" s="18" t="n"/>
+      <c r="K32" s="18" t="n"/>
+      <c r="L32" s="18" t="n"/>
+      <c r="M32" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A27:M27"/>
+    <mergeCell ref="A32:M32"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A31:J31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -4474,6 +4711,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Living room: GKB soffit underside, NaturHeld 40 side face; refresh #69 study note
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>38.27</v>
+        <v>25.65</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>42.1</v>
+        <v>28.22</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>12.76 m² × 3,0 = 38.3 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
+          <t>8.55 m² × 3,0 = 25.7 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>31.89</v>
+        <v>21.38</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>35.08</v>
+        <v>23.52</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>12.76 m² × 2,5 = 31.9 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
+          <t>8.55 m² × 2,5 = 21.4 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>12.76</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1808,13 +1808,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>14.29</v>
+        <v>9.58</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3801</v>
+        <v>2548</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.78</v>
+        <v>1.9</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1.95</v>
+        <v>2.09</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1918,13 +1918,13 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>20.3</v>
+        <v>20.9</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>14648</v>
+        <v>13412</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -3126,7 +3126,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>251.28</v>
+        <v>238.66</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>276.4</v>
+        <v>262.52</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Šikminy+kastlík 83.76 m² → 251.3 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
+          <t>Šikminy+kastlík 79.55 m² → 238.7 kg; objednat 15× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>209.4</v>
+        <v>198.88</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>230.34</v>
+        <v>218.77</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>209.4 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
+          <t>198.9 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>12.76</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -3353,13 +3353,13 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>14.29</v>
+        <v>9.58</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>3801</v>
+        <v>2548</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Kastlík, svislý líc (podhled je GKB).</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
+          <t>Sádrokarton GKB/RF 12,5 (basstrapy + podhled kastlíku)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3688,7 +3688,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>18.19</v>
+        <v>22.44</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3701,13 +3701,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>20.37</v>
+        <v>25.13</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>1956</v>
+        <v>2413</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Štíty 18.19 m² + podhled kastlíku nad skříněmi 4.25 m².</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="F14" s="9" t="n">
-        <v>231.9</v>
+        <v>232.5</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
@@ -3758,13 +3758,13 @@
         </is>
       </c>
       <c r="I14" s="9" t="n">
-        <v>255.1</v>
+        <v>255.7</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>7452</v>
+        <v>7469</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>5.5</v>
+        <v>5.63</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="I23" s="6" t="n">
-        <v>6.05</v>
+        <v>6.19</v>
       </c>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
+          <t>Kastlík 1.90 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       <c r="I31" s="15" t="n"/>
       <c r="J31" s="15" t="n"/>
       <c r="K31" s="16" t="n">
-        <v>96269</v>
+        <v>95490</v>
       </c>
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>12.76 m²</t>
+          <t>8.55 m²</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Living room: room-wave study with domestic sofa (#69) + GKB soffit underside (#71)
Consolidates draft #69 (room-wave study, domestic sofa, asymmetric
NaturHeld comparison) rebased onto main (#68/#70 geometry wins: NH 60
left / 100 right, 2x GKF right, h_start 3184.8, no CD shift).

Soffit: underside is plain GKB 12.5 (`soffit_gkb`), side face stays
NaturHeld 140 40 mm + StoSilent. 1D acoustics mix side (NH stack) and
underside (GKB on soffit wool + duct air) by area. BOM: NH 40 and
StoSilent now side face only; GKB line includes the soffit underside.

Supersedes #69. The archived wave study doc has a status note; its
tables were not re-run (roomwave still treats the soffit as NH).

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Bob <petrsima+bob@mail.grokbot.com>
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>38.27</v>
+        <v>25.65</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>42.1</v>
+        <v>28.22</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>12.76 m² × 3,0 = 38.3 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
+          <t>8.55 m² × 3,0 = 25.7 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>31.89</v>
+        <v>21.38</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>35.08</v>
+        <v>23.52</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>12.76 m² × 2,5 = 31.9 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
+          <t>8.55 m² × 2,5 = 21.4 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>12.76</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1808,13 +1808,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>14.29</v>
+        <v>9.58</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3801</v>
+        <v>2548</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.78</v>
+        <v>1.9</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1.95</v>
+        <v>2.09</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1918,13 +1918,13 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>20.3</v>
+        <v>20.9</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>14648</v>
+        <v>13412</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -3126,7 +3126,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>251.28</v>
+        <v>238.66</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>276.4</v>
+        <v>262.52</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Šikminy+kastlík 83.76 m² → 251.3 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
+          <t>Šikminy+kastlík 79.55 m² → 238.7 kg; objednat 15× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>209.4</v>
+        <v>198.88</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>230.34</v>
+        <v>218.77</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>209.4 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
+          <t>198.9 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>12.76</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -3353,13 +3353,13 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>14.29</v>
+        <v>9.58</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>3801</v>
+        <v>2548</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Kastlík, svislý líc (podhled je GKB).</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
+          <t>Sádrokarton GKB/RF 12,5 (basstrapy + podhled kastlíku)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3688,7 +3688,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>18.19</v>
+        <v>22.44</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3701,13 +3701,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>20.37</v>
+        <v>25.13</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>1956</v>
+        <v>2413</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Štíty 18.19 m² + podhled kastlíku nad skříněmi 4.25 m².</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="F14" s="9" t="n">
-        <v>231.9</v>
+        <v>232.5</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
@@ -3758,13 +3758,13 @@
         </is>
       </c>
       <c r="I14" s="9" t="n">
-        <v>255.1</v>
+        <v>255.7</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>7452</v>
+        <v>7469</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>5.5</v>
+        <v>5.63</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="I23" s="6" t="n">
-        <v>6.05</v>
+        <v>6.19</v>
       </c>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
+          <t>Kastlík 1.90 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       <c r="I31" s="15" t="n"/>
       <c r="J31" s="15" t="n"/>
       <c r="K31" s="16" t="n">
-        <v>96269</v>
+        <v>95490</v>
       </c>
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>12.76 m²</t>
+          <t>8.55 m²</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
obyvak: eave details — left GKF on UD to wall plate, continuous vapour brake taped to plaster, right GKF bears on soffit lid
- Left eave: bent UD screwed to the plate cheek, GKF ends in it, NaturHeld bears on the wall,
  vapour brake runs down past the plate with a slack loop and is taped to wall plaster;
  acrylic bead at the planned corner cut. New detail model obyvak_eave_left.
- Vapour brake modelled as one continuous layer eave to eave.
- Right eave: slope GKF cut level and bearing on the lid (no gap, no acrylic joint),
  lid CD moved under the outer GKF plane, NaturHeld level toe so wool fills to the boards.
- obyvak_joint now clipped from the section (shared obyvak_detail helper).
- BOM: Jutafol eave runs, left eave UD, bond tape/mastic, acrylic.
- Tests updated.
</commit_message>
<xml_diff>
--- a/docs/obyvak-skladba-materialu.xlsx
+++ b/docs/obyvak-skladba-materialu.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>71</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -827,13 +827,13 @@
         </is>
       </c>
       <c r="I6" s="9" t="n">
-        <v>78.09999999999999</v>
+        <v>88.81</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>35.73</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2791</v>
+        <v>3173</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m². S rezervou 10 % ≈ 78.1 m² ≈ 2× role 75 m². Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
+          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m² + přesahy u okapů 9.74 m² (877 mm × 11.1 m: vlevo dolů přes pozednici se smyčkou na omítku, vpravo přes víko kastlíku na omítku skříní). S rezervou 10 % ≈ 88.8 m² ≈ 2× role 75 m². Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Second layer on the road-side slope for road noise. Joints staggered against the first layer. Same 3 mm acrylic joint at the soffit.</t>
+          <t>Second layer on the road-side slope for road noise. Joints staggered against the first layer. Both layers cut level and bear on the soffit lid (no gap).</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
       <c r="K19" s="16" t="n">
-        <v>57101</v>
+        <v>57484</v>
       </c>
       <c r="L19" s="15" t="n"/>
       <c r="M19" s="15" t="n"/>
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>4.98</v>
+        <v>5.44</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1975,13 +1975,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>5.58</v>
+        <v>6.09</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>646</v>
+        <v>706</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>1 závěs na krokev na rostovém CD. Svěšení 406 mm.</t>
+          <t>1 závěs na krokev na rostovém CD. Svěšení 390 mm.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>13412</v>
+        <v>13472</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2997,7 +2997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>71</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3410,13 +3410,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>78.09999999999999</v>
+        <v>88.81</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>35.73</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>2791</v>
+        <v>3173</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
+          <t>Šikminy 71.00 m² + okapy 9.74 m² (+10 % ≈ 88.8 m²). Nad CD, pod vlnou; na obou okapech dolů na omítku se smyčkou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>75.98</v>
+        <v>76.44</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>85.09999999999999</v>
+        <v>85.61</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>9861</v>
+        <v>9921</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina + kastlík. Svěšení šikminy 309 mm, kastlík 406 mm. Load with 2× GKF ≈ 22 kg per hanger point (was ≈ 17 kg); Nonius load class 0.40 kN, so OK.</t>
+          <t>Pravá šikmina + kastlík. Svěšení šikminy 309 mm, kastlík 390 mm. Load with 2× GKF ≈ 22 kg per hanger point (was ≈ 17 kg); Nonius load class 0.40 kN, so OK.</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. Spára akryl + páska 10.46 bm.</t>
+          <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. GKF šikminy dosedá na víko kastlíku bez spáry.</t>
         </is>
       </c>
     </row>
@@ -4348,31 +4348,33 @@
       </c>
     </row>
     <row r="25" ht="52" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>16</v>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>15b</t>
+        </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Zavětrovací pásky 40×2</t>
+          <t>UD 28×27 na pozednici (levý okap)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Ocelová páska</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>Rigips UD 28/27, ohnutá pásnice</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>40×2</t>
+          <t>28×27 · vrut do dřeva 3,5×35 @ 300 mm</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>32.6</v>
+        <v>11.1</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -4385,51 +4387,53 @@
         </is>
       </c>
       <c r="I25" s="6" t="n">
-        <v>35.8</v>
+        <v>12.2</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>25</v>
+        <v>29.21</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>896</v>
+        <v>357</v>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>orientační ocelová páska 40×2</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: přesný typ.</t>
+          <t>Konec GKF levé šikminy. Ohnutá pásnice přišroubovaná na čelo pozednice. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="4" t="n">
-        <v>17</v>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>15c</t>
+        </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>Napojení parozábrany na omítku</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>Lepicí páska / tmel</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>JUTAFOL MASTIC + páska (typ Contega / Orcon)</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>oba okapy</t>
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>31.4</v>
+        <v>22.2</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -4438,59 +4442,57 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I26" s="6" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="J26" s="12" t="n">
-        <v>180</v>
-      </c>
-      <c r="K26" s="13" t="n">
-        <v>6099</v>
-      </c>
+        <v>24.4</v>
+      </c>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>Vlevo: fólie dolů přes pozednici, volná smyčka, nalepit a přelepit na omítku zdi. Vpravo: přes víko kastlíku dolů, smyčka, na omítku skříní. Lepená plocha vlevo je krátká (~27 mm) — použít lepidlo pro omítky.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>18</v>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>15d</t>
+        </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>Akryl v koutě (plánovaná spára)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>Akrylový tmel</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Akryl přetíratelný</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>levý kout stěna/šikmina</t>
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>17</v>
+        <v>11.1</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -4499,51 +4501,47 @@
         </is>
       </c>
       <c r="I27" s="6" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="J27" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="K27" s="13" t="n">
-        <v>150</v>
-      </c>
+        <v>12.2</v>
+      </c>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Kout zeď / GKF levé šikminy je plánovaný řez, uzavřený akrylem.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="52" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>20.9</v>
+        <v>32.6</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -4556,143 +4554,314 @@
         </is>
       </c>
       <c r="I28" s="6" t="n">
-        <v>23</v>
+        <v>35.8</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="K28" s="13" t="n">
-        <v>1265</v>
+        <v>896</v>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="52" customHeight="1">
       <c r="A29" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Spirála Ø160</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>VZT potrubí</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Výrobce VZT dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Ø160</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="K29" s="13" t="n">
+        <v>6099</v>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>orientační spirála Ø160 pozink</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>3 trasy v kastlíku.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="52" customHeight="1">
+      <c r="A30" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J30" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K30" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J31" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K31" s="13" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1">
+      <c r="A32" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="F32" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I29" s="6" t="n">
+      <c r="I32" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J32" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K29" s="13" t="n">
+      <c r="K32" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="16" t="n">
-        <v>95490</v>
-      </c>
-      <c r="L31" s="15" t="n"/>
-      <c r="M31" s="15" t="n"/>
-    </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="B32" s="18" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="18" t="n"/>
-      <c r="L32" s="18" t="n"/>
-      <c r="M32" s="18" t="n"/>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="15" t="n"/>
+      <c r="I34" s="15" t="n"/>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="16" t="n">
+        <v>96289</v>
+      </c>
+      <c r="L34" s="15" t="n"/>
+      <c r="M34" s="15" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty; Napojení parozábrany na omítku; Akryl v koutě (plánovaná spára)</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="n"/>
+      <c r="C35" s="18" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="18" t="n"/>
+      <c r="L35" s="18" t="n"/>
+      <c r="M35" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="A33:M33"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A34:J34"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>

</xml_diff>